<commit_message>
Adding personal Lists file
</commit_message>
<xml_diff>
--- a/Comedy_Whitelist.xlsx
+++ b/Comedy_Whitelist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bigba\aa Personal Projects\Letterboxd-List-Scraping\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B96D3FFA-3D9F-49A8-8911-81864113D2C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB0623FF-6D56-4BAE-84D2-0D19C05A4F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1740" yWindow="1740" windowWidth="14400" windowHeight="8170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="294">
   <si>
     <t>Title</t>
   </si>
@@ -874,9 +874,6 @@
     <t>https://letterboxd.com/film/chris-fleming-showpig/</t>
   </si>
   <si>
-    <t>Yes</t>
-  </si>
-  <si>
     <t>https://letterboxd.com/film/daniel-sloss-socio/</t>
   </si>
   <si>
@@ -893,6 +890,18 @@
   </si>
   <si>
     <t>https://letterboxd.com/film/eddie-izzard-definite-article/</t>
+  </si>
+  <si>
+    <t>Stewart Lee, Basic Lee: Live at The Lowry</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/stewart-lee-basic-lee-live-at-the-lowry/</t>
+  </si>
+  <si>
+    <t>Doug Stanhope: No Refunds</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/doug-stanhope-no-refunds/</t>
   </si>
 </sst>
 </file>
@@ -1266,7 +1275,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E124"/>
+  <dimension ref="A1:D126"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
@@ -2837,7 +2846,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>266</v>
       </c>
@@ -2851,7 +2860,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>268</v>
       </c>
@@ -2865,7 +2874,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>270</v>
       </c>
@@ -2879,7 +2888,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>272</v>
       </c>
@@ -2893,7 +2902,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>274</v>
       </c>
@@ -2907,7 +2916,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>276</v>
       </c>
@@ -2921,7 +2930,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>278</v>
       </c>
@@ -2935,7 +2944,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>280</v>
       </c>
@@ -2949,7 +2958,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>282</v>
       </c>
@@ -2963,9 +2972,9 @@
         <v>283</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B122">
         <v>2022</v>
@@ -2974,15 +2983,12 @@
         <v>1054105</v>
       </c>
       <c r="D122" s="2" t="s">
-        <v>285</v>
-      </c>
-      <c r="E122" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B123">
         <v>2026</v>
@@ -2991,12 +2997,12 @@
         <v>1723570</v>
       </c>
       <c r="D123" s="2" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A124" t="s">
         <v>288</v>
-      </c>
-    </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A124" t="s">
-        <v>289</v>
       </c>
       <c r="B124">
         <v>1996</v>
@@ -3005,7 +3011,35 @@
         <v>13588</v>
       </c>
       <c r="D124" s="2" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A125" t="s">
         <v>290</v>
+      </c>
+      <c r="B125">
+        <v>2024</v>
+      </c>
+      <c r="C125">
+        <v>1237421</v>
+      </c>
+      <c r="D125" s="2" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A126" t="s">
+        <v>292</v>
+      </c>
+      <c r="B126">
+        <v>2007</v>
+      </c>
+      <c r="C126">
+        <v>18362</v>
+      </c>
+      <c r="D126" s="2" t="s">
+        <v>293</v>
       </c>
     </row>
   </sheetData>
@@ -3015,6 +3049,8 @@
     <hyperlink ref="D122" r:id="rId3" xr:uid="{47150D12-8DC3-428F-AB07-31014E62FB05}"/>
     <hyperlink ref="D123" r:id="rId4" xr:uid="{447BDA79-8975-419D-95B9-8B8FD5823A2D}"/>
     <hyperlink ref="D124" r:id="rId5" xr:uid="{F2FA2C83-21B1-492F-A27F-DD32C1868DD7}"/>
+    <hyperlink ref="D125" r:id="rId6" xr:uid="{1219CF77-A5AA-4862-8376-1B14DCBECE2C}"/>
+    <hyperlink ref="D126" r:id="rId7" xr:uid="{294E2AD0-2975-4BEB-814D-31754A2517A7}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>